<commit_message>
Add folder skeleton markers and updated session summary
</commit_message>
<xml_diff>
--- a/resources/reference/orthologue_domain_summary.xlsx
+++ b/resources/reference/orthologue_domain_summary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juliethmurillo/Documents/GitHub/aviced_bioinformatics/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juliethmurillo/Documents/GitHub/aviced_bioinformatics/resources/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84FB50E-6778-204F-8E22-02E12349F3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51EC8F5A-9611-8145-99E9-4DCF822B67E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -992,7 +992,7 @@
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="50.1640625" customWidth="1"/>
     <col min="11" max="11" width="27.5" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" customWidth="1"/>
+    <col min="12" max="12" width="35" customWidth="1"/>
     <col min="13" max="13" width="18" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
     <col min="15" max="17" width="45" customWidth="1"/>
@@ -1375,7 +1375,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="91" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="65" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>37</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="39" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" ht="65" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>68</v>
       </c>
@@ -1878,7 +1878,7 @@
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
     </row>
-    <row r="21" spans="1:17" ht="39" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" ht="65" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
@@ -2822,7 +2822,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="26" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>114</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="65" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17" ht="52" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>120</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="1:17" ht="52" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:17" ht="104" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>125</v>
       </c>
@@ -3705,7 +3705,7 @@
       <c r="P61" s="2"/>
       <c r="Q61" s="2"/>
     </row>
-    <row r="62" spans="1:17" ht="52" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:17" ht="91" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>157</v>
       </c>
@@ -3750,7 +3750,7 @@
       <c r="P62" s="2"/>
       <c r="Q62" s="2"/>
     </row>
-    <row r="63" spans="1:17" ht="52" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:17" ht="39" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>162</v>
       </c>

</xml_diff>